<commit_message>
Refactor uploadVoters and uploadDraftVoters API methods to use queryFn with improved error handling and timeout management
</commit_message>
<xml_diff>
--- a/public/Voter_Sample_Data.xlsx
+++ b/public/Voter_Sample_Data.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AZ1"/>
+  <dimension ref="A1:CP1"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -451,169 +451,337 @@
     <col min="50" max="50" width="20.83203125" customWidth="1"/>
     <col min="51" max="51" width="20.83203125" customWidth="1"/>
     <col min="52" max="52" width="20.83203125" customWidth="1"/>
+    <col min="53" max="53" width="20.83203125" customWidth="1"/>
+    <col min="54" max="54" width="20.83203125" customWidth="1"/>
+    <col min="55" max="55" width="20.83203125" customWidth="1"/>
+    <col min="56" max="56" width="20.83203125" customWidth="1"/>
+    <col min="57" max="57" width="20.83203125" customWidth="1"/>
+    <col min="58" max="58" width="20.83203125" customWidth="1"/>
+    <col min="59" max="59" width="20.83203125" customWidth="1"/>
+    <col min="60" max="60" width="20.83203125" customWidth="1"/>
+    <col min="61" max="61" width="20.83203125" customWidth="1"/>
+    <col min="62" max="62" width="20.83203125" customWidth="1"/>
+    <col min="63" max="63" width="20.83203125" customWidth="1"/>
+    <col min="64" max="64" width="20.83203125" customWidth="1"/>
+    <col min="65" max="65" width="20.83203125" customWidth="1"/>
+    <col min="66" max="66" width="20.83203125" customWidth="1"/>
+    <col min="67" max="67" width="20.83203125" customWidth="1"/>
+    <col min="68" max="68" width="20.83203125" customWidth="1"/>
+    <col min="69" max="69" width="20.83203125" customWidth="1"/>
+    <col min="70" max="70" width="20.83203125" customWidth="1"/>
+    <col min="71" max="71" width="20.83203125" customWidth="1"/>
+    <col min="72" max="72" width="20.83203125" customWidth="1"/>
+    <col min="73" max="73" width="20.83203125" customWidth="1"/>
+    <col min="74" max="74" width="20.83203125" customWidth="1"/>
+    <col min="75" max="75" width="20.83203125" customWidth="1"/>
+    <col min="76" max="76" width="20.83203125" customWidth="1"/>
+    <col min="77" max="77" width="20.83203125" customWidth="1"/>
+    <col min="78" max="78" width="20.83203125" customWidth="1"/>
+    <col min="79" max="79" width="20.83203125" customWidth="1"/>
+    <col min="80" max="80" width="20.83203125" customWidth="1"/>
+    <col min="81" max="81" width="20.83203125" customWidth="1"/>
+    <col min="82" max="82" width="20.83203125" customWidth="1"/>
+    <col min="83" max="83" width="20.83203125" customWidth="1"/>
+    <col min="84" max="84" width="20.83203125" customWidth="1"/>
+    <col min="85" max="85" width="20.83203125" customWidth="1"/>
+    <col min="86" max="86" width="20.83203125" customWidth="1"/>
+    <col min="87" max="87" width="20.83203125" customWidth="1"/>
+    <col min="88" max="88" width="20.83203125" customWidth="1"/>
+    <col min="89" max="89" width="20.83203125" customWidth="1"/>
+    <col min="90" max="90" width="20.83203125" customWidth="1"/>
+    <col min="91" max="91" width="20.83203125" customWidth="1"/>
+    <col min="92" max="92" width="20.83203125" customWidth="1"/>
+    <col min="93" max="93" width="20.83203125" customWidth="1"/>
+    <col min="94" max="94" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>AC_NO</v>
+        <v>ac_no</v>
       </c>
       <c r="B1" t="str">
-        <v>PART_NO</v>
+        <v>ac_name_en</v>
       </c>
       <c r="C1" t="str">
-        <v>SECTION_NO</v>
+        <v>ac_name_v1</v>
       </c>
       <c r="D1" t="str">
-        <v>SLNOINPART</v>
+        <v>part_no</v>
       </c>
       <c r="E1" t="str">
-        <v>HOUSE_NO_EN</v>
+        <v>part_name_en</v>
       </c>
       <c r="F1" t="str">
-        <v>HOUSE_NO_V1</v>
+        <v>part_name_v1</v>
       </c>
       <c r="G1" t="str">
-        <v>Voter_FULL_NAME_EN</v>
+        <v>section_no</v>
       </c>
       <c r="H1" t="str">
-        <v>LAST_NAME_EN</v>
+        <v>section_name_en</v>
       </c>
       <c r="I1" t="str">
-        <v>Voter_Full_NAME_V1</v>
+        <v>section_name_v1</v>
       </c>
       <c r="J1" t="str">
-        <v>LASTNAME_V1</v>
+        <v>sl_no_in_part</v>
       </c>
       <c r="K1" t="str">
-        <v>RLN_TYPE</v>
+        <v>house_no_eng</v>
       </c>
       <c r="L1" t="str">
-        <v>RLN_FM_NM_EN</v>
+        <v>house_no_hi</v>
       </c>
       <c r="M1" t="str">
-        <v>RLN_L_NM_EN</v>
+        <v>house_no</v>
       </c>
       <c r="N1" t="str">
-        <v>RLN_FM_NM_V1</v>
+        <v>voter_full_name_en</v>
       </c>
       <c r="O1" t="str">
-        <v>RLN_L_NM_V1</v>
+        <v>voter_last_name_en</v>
       </c>
       <c r="P1" t="str">
-        <v>EPIC_NO</v>
+        <v>voter_full_name_hi</v>
       </c>
       <c r="Q1" t="str">
-        <v>GENDER</v>
+        <v>voter_last_name_hi</v>
       </c>
       <c r="R1" t="str">
-        <v>AGE</v>
+        <v>voter_name</v>
       </c>
       <c r="S1" t="str">
-        <v>DOB</v>
+        <v>voter_name_hi</v>
       </c>
       <c r="T1" t="str">
-        <v>MOBILE_NO</v>
+        <v>relative_full_name_en</v>
       </c>
       <c r="U1" t="str">
-        <v>AC_NAME_EN</v>
+        <v>relative_last_name_en</v>
       </c>
       <c r="V1" t="str">
-        <v>AC_NAME_V1</v>
+        <v>relative_full_name_hi</v>
       </c>
       <c r="W1" t="str">
-        <v>PART_NAME_EN</v>
+        <v>relative_last_name_hi</v>
       </c>
       <c r="X1" t="str">
-        <v>PART_NAME_V1</v>
+        <v>relation</v>
       </c>
       <c r="Y1" t="str">
-        <v>SECTION_NAME_EN</v>
+        <v>father_name</v>
       </c>
       <c r="Z1" t="str">
-        <v>SECTION_NAME_V1</v>
+        <v>father_name_en</v>
       </c>
       <c r="AA1" t="str">
-        <v>Polling _Station_Name_EN</v>
+        <v>father_name_hi</v>
       </c>
       <c r="AB1" t="str">
-        <v>Polling _Station_Name_V1</v>
+        <v>voter_id_epic_no</v>
       </c>
       <c r="AC1" t="str">
-        <v>Polling_Station_BUILDING_NAME_EN</v>
+        <v>epic_no</v>
       </c>
       <c r="AD1" t="str">
-        <v>Polling_Station_BUILDING_NAME_V1</v>
+        <v>gender</v>
       </c>
       <c r="AE1" t="str">
-        <v>MOBILE_NO_2</v>
+        <v>age</v>
       </c>
       <c r="AF1" t="str">
-        <v>MOBILE_NO_3</v>
+        <v>voter_dob</v>
       </c>
       <c r="AG1" t="str">
-        <v>MOBILE_NO_4</v>
+        <v>birth_date_eng</v>
       </c>
       <c r="AH1" t="str">
-        <v>STATE_Code</v>
+        <v>contact_number1</v>
       </c>
       <c r="AI1" t="str">
-        <v>state_name_en</v>
+        <v>contact_number2</v>
       </c>
       <c r="AJ1" t="str">
-        <v>state_name_V1</v>
+        <v>contact_number3</v>
       </c>
       <c r="AK1" t="str">
+        <v>contact_number4</v>
+      </c>
+      <c r="AL1" t="str">
+        <v>mobile_no</v>
+      </c>
+      <c r="AM1" t="str">
+        <v>mobile_no_2</v>
+      </c>
+      <c r="AN1" t="str">
+        <v>mobile_no_3</v>
+      </c>
+      <c r="AO1" t="str">
+        <v>mobile_no_4</v>
+      </c>
+      <c r="AP1" t="str">
+        <v>state_code</v>
+      </c>
+      <c r="AQ1" t="str">
+        <v>state_name_eng</v>
+      </c>
+      <c r="AR1" t="str">
+        <v>state_name_hi</v>
+      </c>
+      <c r="AS1" t="str">
         <v>distt_name_en</v>
       </c>
-      <c r="AL1" t="str">
-        <v>distt_name_V1</v>
-      </c>
-      <c r="AM1" t="str">
-        <v>PC_LS_NO</v>
-      </c>
-      <c r="AN1" t="str">
-        <v>PC_LS_NAME_EN</v>
-      </c>
-      <c r="AO1" t="str">
-        <v>PC_LS_NAME_V1</v>
-      </c>
-      <c r="AP1" t="str">
+      <c r="AT1" t="str">
+        <v>distt_name_v1</v>
+      </c>
+      <c r="AU1" t="str">
+        <v>distt_name_hi</v>
+      </c>
+      <c r="AV1" t="str">
+        <v>pc_no</v>
+      </c>
+      <c r="AW1" t="str">
+        <v>pc_name_en</v>
+      </c>
+      <c r="AX1" t="str">
+        <v>pc_name_v1</v>
+      </c>
+      <c r="AY1" t="str">
+        <v>pc_name_hi</v>
+      </c>
+      <c r="AZ1" t="str">
         <v>town_village_name_eng</v>
       </c>
-      <c r="AQ1" t="str">
-        <v>town_village_name_v1</v>
-      </c>
-      <c r="AR1" t="str">
+      <c r="BA1" t="str">
+        <v>town_village_name_hi</v>
+      </c>
+      <c r="BB1" t="str">
         <v>ward_no</v>
       </c>
-      <c r="AS1" t="str">
+      <c r="BC1" t="str">
         <v>ward_elec_id</v>
       </c>
-      <c r="AT1" t="str">
-        <v>Ward_name_En</v>
-      </c>
-      <c r="AU1" t="str">
-        <v>Ward_name_V1</v>
-      </c>
-      <c r="AV1" t="str">
-        <v>Tehsil_EN</v>
-      </c>
-      <c r="AW1" t="str">
-        <v>Tehsil_V1</v>
-      </c>
-      <c r="AX1" t="str">
+      <c r="BD1" t="str">
+        <v>ward_name_en</v>
+      </c>
+      <c r="BE1" t="str">
+        <v>ward_name_v1</v>
+      </c>
+      <c r="BF1" t="str">
+        <v>tehsil_eng</v>
+      </c>
+      <c r="BG1" t="str">
+        <v>tehsil_hi</v>
+      </c>
+      <c r="BH1" t="str">
         <v>police_station_en</v>
       </c>
-      <c r="AY1" t="str">
+      <c r="BI1" t="str">
         <v>police_station_v1</v>
       </c>
-      <c r="AZ1" t="str">
+      <c r="BJ1" t="str">
         <v>pincode</v>
+      </c>
+      <c r="BK1" t="str">
+        <v>ps_name_en</v>
+      </c>
+      <c r="BL1" t="str">
+        <v>ps_name_v1</v>
+      </c>
+      <c r="BM1" t="str">
+        <v>ps_loc_en</v>
+      </c>
+      <c r="BN1" t="str">
+        <v>ps_loc_hin</v>
+      </c>
+      <c r="BO1" t="str">
+        <v>aadhar</v>
+      </c>
+      <c r="BP1" t="str">
+        <v>religion</v>
+      </c>
+      <c r="BQ1" t="str">
+        <v>caste</v>
+      </c>
+      <c r="BR1" t="str">
+        <v>profession_type</v>
+      </c>
+      <c r="BS1" t="str">
+        <v>profession_sub_catg</v>
+      </c>
+      <c r="BT1" t="str">
+        <v>married</v>
+      </c>
+      <c r="BU1" t="str">
+        <v>education</v>
+      </c>
+      <c r="BV1" t="str">
+        <v>shifted</v>
+      </c>
+      <c r="BW1" t="str">
+        <v>shifted_address</v>
+      </c>
+      <c r="BX1" t="str">
+        <v>shifted_country</v>
+      </c>
+      <c r="BY1" t="str">
+        <v>shifted_state</v>
+      </c>
+      <c r="BZ1" t="str">
+        <v>shifted_city</v>
+      </c>
+      <c r="CA1" t="str">
+        <v>staying_outside</v>
+      </c>
+      <c r="CB1" t="str">
+        <v>staying_address</v>
+      </c>
+      <c r="CC1" t="str">
+        <v>staying_country</v>
+      </c>
+      <c r="CD1" t="str">
+        <v>staying_state</v>
+      </c>
+      <c r="CE1" t="str">
+        <v>staying_city</v>
+      </c>
+      <c r="CF1" t="str">
+        <v>labarthi_in_person</v>
+      </c>
+      <c r="CG1" t="str">
+        <v>labarthi_state</v>
+      </c>
+      <c r="CH1" t="str">
+        <v>labarthi_center</v>
+      </c>
+      <c r="CI1" t="str">
+        <v>outside_country</v>
+      </c>
+      <c r="CJ1" t="str">
+        <v>influencer</v>
+      </c>
+      <c r="CK1" t="str">
+        <v>eu_ssr_form_submitted</v>
+      </c>
+      <c r="CL1" t="str">
+        <v>family_id</v>
+      </c>
+      <c r="CM1" t="str">
+        <v>relative_in_part_no</v>
+      </c>
+      <c r="CN1" t="str">
+        <v>relative_sl_in_part</v>
+      </c>
+      <c r="CO1" t="str">
+        <v>expired_alive</v>
+      </c>
+      <c r="CP1" t="str">
+        <v>political_party</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AZ1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:CP1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>